<commit_message>
Update ITA exam archive
</commit_message>
<xml_diff>
--- a/ita_provas/manifest.xlsx
+++ b/ita_provas/manifest.xlsx
@@ -1,22 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c308351cf5a860c7/github_oz/military_sat/ita_provas/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{5672D07B-9D6C-41DE-92D3-5CD0C2281E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Manifest" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -920,35 +913,32 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <sz val="11"/>
-      <name val="Aptos Narrow"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Aptos Narrow"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -960,34 +950,47 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ManifestTable" displayName="ManifestTable" ref="A1:F96" totalsRowShown="0">
+  <autoFilter ref="A1:F96"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="year"/>
+    <tableColumn id="2" name="label"/>
+    <tableColumn id="3" name="path"/>
+    <tableColumn id="4" name="bytes"/>
+    <tableColumn id="5" name="sha256"/>
+    <tableColumn id="6" name="source_url"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -997,44 +1000,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -1061,32 +1064,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -1113,24 +1098,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1142,200 +1109,204 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F96"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="45" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="68" customWidth="1"/>
-    <col min="6" max="6" width="65" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="45.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="68.7109375" customWidth="1"/>
+    <col min="6" max="6" width="65.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A2">
+    <row r="2" spans="1:6">
+      <c r="A2" s="1">
         <v>2026</v>
       </c>
       <c r="B2" t="s">
@@ -1350,12 +1321,12 @@
       <c r="E2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A3">
+    <row r="3" spans="1:6">
+      <c r="A3" s="1">
         <v>2026</v>
       </c>
       <c r="B3" t="s">
@@ -1370,12 +1341,12 @@
       <c r="E3" t="s">
         <v>12</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A4">
+    <row r="4" spans="1:6">
+      <c r="A4" s="1">
         <v>2026</v>
       </c>
       <c r="B4" t="s">
@@ -1390,12 +1361,12 @@
       <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A5">
+    <row r="5" spans="1:6">
+      <c r="A5" s="1">
         <v>2026</v>
       </c>
       <c r="B5" t="s">
@@ -1410,12 +1381,12 @@
       <c r="E5" t="s">
         <v>20</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A6">
+    <row r="6" spans="1:6">
+      <c r="A6" s="1">
         <v>2026</v>
       </c>
       <c r="B6" t="s">
@@ -1430,12 +1401,12 @@
       <c r="E6" t="s">
         <v>24</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A7">
+    <row r="7" spans="1:6">
+      <c r="A7" s="1">
         <v>2025</v>
       </c>
       <c r="B7" t="s">
@@ -1450,12 +1421,12 @@
       <c r="E7" t="s">
         <v>27</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A8">
+    <row r="8" spans="1:6">
+      <c r="A8" s="1">
         <v>2025</v>
       </c>
       <c r="B8" t="s">
@@ -1470,12 +1441,12 @@
       <c r="E8" t="s">
         <v>30</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A9">
+    <row r="9" spans="1:6">
+      <c r="A9" s="1">
         <v>2025</v>
       </c>
       <c r="B9" t="s">
@@ -1490,12 +1461,12 @@
       <c r="E9" t="s">
         <v>33</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A10">
+    <row r="10" spans="1:6">
+      <c r="A10" s="1">
         <v>2025</v>
       </c>
       <c r="B10" t="s">
@@ -1510,12 +1481,12 @@
       <c r="E10" t="s">
         <v>36</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A11">
+    <row r="11" spans="1:6">
+      <c r="A11" s="1">
         <v>2025</v>
       </c>
       <c r="B11" t="s">
@@ -1530,12 +1501,12 @@
       <c r="E11" t="s">
         <v>39</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A12">
+    <row r="12" spans="1:6">
+      <c r="A12" s="1">
         <v>2024</v>
       </c>
       <c r="B12" t="s">
@@ -1550,12 +1521,12 @@
       <c r="E12" t="s">
         <v>42</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A13">
+    <row r="13" spans="1:6">
+      <c r="A13" s="1">
         <v>2024</v>
       </c>
       <c r="B13" t="s">
@@ -1570,12 +1541,12 @@
       <c r="E13" t="s">
         <v>45</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="3" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A14">
+    <row r="14" spans="1:6">
+      <c r="A14" s="1">
         <v>2024</v>
       </c>
       <c r="B14" t="s">
@@ -1590,12 +1561,12 @@
       <c r="E14" t="s">
         <v>48</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A15">
+    <row r="15" spans="1:6">
+      <c r="A15" s="1">
         <v>2024</v>
       </c>
       <c r="B15" t="s">
@@ -1610,12 +1581,12 @@
       <c r="E15" t="s">
         <v>51</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A16">
+    <row r="16" spans="1:6">
+      <c r="A16" s="1">
         <v>2024</v>
       </c>
       <c r="B16" t="s">
@@ -1630,12 +1601,12 @@
       <c r="E16" t="s">
         <v>55</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A17">
+    <row r="17" spans="1:6">
+      <c r="A17" s="1">
         <v>2023</v>
       </c>
       <c r="B17" t="s">
@@ -1650,12 +1621,12 @@
       <c r="E17" t="s">
         <v>58</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A18">
+    <row r="18" spans="1:6">
+      <c r="A18" s="1">
         <v>2023</v>
       </c>
       <c r="B18" t="s">
@@ -1670,12 +1641,12 @@
       <c r="E18" t="s">
         <v>61</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A19">
+    <row r="19" spans="1:6">
+      <c r="A19" s="1">
         <v>2023</v>
       </c>
       <c r="B19" t="s">
@@ -1690,12 +1661,12 @@
       <c r="E19" t="s">
         <v>64</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A20">
+    <row r="20" spans="1:6">
+      <c r="A20" s="1">
         <v>2023</v>
       </c>
       <c r="B20" t="s">
@@ -1710,12 +1681,12 @@
       <c r="E20" t="s">
         <v>67</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A21">
+    <row r="21" spans="1:6">
+      <c r="A21" s="1">
         <v>2023</v>
       </c>
       <c r="B21" t="s">
@@ -1730,12 +1701,12 @@
       <c r="E21" t="s">
         <v>70</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A22">
+    <row r="22" spans="1:6">
+      <c r="A22" s="1">
         <v>2022</v>
       </c>
       <c r="B22" t="s">
@@ -1750,12 +1721,12 @@
       <c r="E22" t="s">
         <v>73</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="3" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A23">
+    <row r="23" spans="1:6">
+      <c r="A23" s="1">
         <v>2022</v>
       </c>
       <c r="B23" t="s">
@@ -1770,12 +1741,12 @@
       <c r="E23" t="s">
         <v>76</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A24">
+    <row r="24" spans="1:6">
+      <c r="A24" s="1">
         <v>2022</v>
       </c>
       <c r="B24" t="s">
@@ -1790,12 +1761,12 @@
       <c r="E24" t="s">
         <v>79</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A25">
+    <row r="25" spans="1:6">
+      <c r="A25" s="1">
         <v>2022</v>
       </c>
       <c r="B25" t="s">
@@ -1810,12 +1781,12 @@
       <c r="E25" t="s">
         <v>82</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A26">
+    <row r="26" spans="1:6">
+      <c r="A26" s="1">
         <v>2022</v>
       </c>
       <c r="B26" t="s">
@@ -1830,12 +1801,12 @@
       <c r="E26" t="s">
         <v>85</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A27">
+    <row r="27" spans="1:6">
+      <c r="A27" s="1">
         <v>2021</v>
       </c>
       <c r="B27" t="s">
@@ -1850,12 +1821,12 @@
       <c r="E27" t="s">
         <v>88</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="3" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A28">
+    <row r="28" spans="1:6">
+      <c r="A28" s="1">
         <v>2021</v>
       </c>
       <c r="B28" t="s">
@@ -1870,12 +1841,12 @@
       <c r="E28" t="s">
         <v>91</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="3" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A29">
+    <row r="29" spans="1:6">
+      <c r="A29" s="1">
         <v>2021</v>
       </c>
       <c r="B29" t="s">
@@ -1890,12 +1861,12 @@
       <c r="E29" t="s">
         <v>94</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A30">
+    <row r="30" spans="1:6">
+      <c r="A30" s="1">
         <v>2021</v>
       </c>
       <c r="B30" t="s">
@@ -1910,12 +1881,12 @@
       <c r="E30" t="s">
         <v>97</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="3" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A31">
+    <row r="31" spans="1:6">
+      <c r="A31" s="1">
         <v>2021</v>
       </c>
       <c r="B31" t="s">
@@ -1930,12 +1901,12 @@
       <c r="E31" t="s">
         <v>100</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A32">
+    <row r="32" spans="1:6">
+      <c r="A32" s="1">
         <v>2020</v>
       </c>
       <c r="B32" t="s">
@@ -1950,12 +1921,12 @@
       <c r="E32" t="s">
         <v>103</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A33">
+    <row r="33" spans="1:6">
+      <c r="A33" s="1">
         <v>2020</v>
       </c>
       <c r="B33" t="s">
@@ -1970,12 +1941,12 @@
       <c r="E33" t="s">
         <v>106</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="3" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A34">
+    <row r="34" spans="1:6">
+      <c r="A34" s="1">
         <v>2020</v>
       </c>
       <c r="B34" t="s">
@@ -1990,12 +1961,12 @@
       <c r="E34" t="s">
         <v>109</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34" s="3" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A35">
+    <row r="35" spans="1:6">
+      <c r="A35" s="1">
         <v>2020</v>
       </c>
       <c r="B35" t="s">
@@ -2010,12 +1981,12 @@
       <c r="E35" t="s">
         <v>112</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="3" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A36">
+    <row r="36" spans="1:6">
+      <c r="A36" s="1">
         <v>2020</v>
       </c>
       <c r="B36" t="s">
@@ -2030,12 +2001,12 @@
       <c r="E36" t="s">
         <v>115</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F36" s="3" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A37">
+    <row r="37" spans="1:6">
+      <c r="A37" s="1">
         <v>2019</v>
       </c>
       <c r="B37" t="s">
@@ -2050,12 +2021,12 @@
       <c r="E37" t="s">
         <v>118</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" s="3" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A38">
+    <row r="38" spans="1:6">
+      <c r="A38" s="1">
         <v>2019</v>
       </c>
       <c r="B38" t="s">
@@ -2070,12 +2041,12 @@
       <c r="E38" t="s">
         <v>121</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" s="3" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A39">
+    <row r="39" spans="1:6">
+      <c r="A39" s="1">
         <v>2019</v>
       </c>
       <c r="B39" t="s">
@@ -2090,12 +2061,12 @@
       <c r="E39" t="s">
         <v>124</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39" s="3" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A40">
+    <row r="40" spans="1:6">
+      <c r="A40" s="1">
         <v>2019</v>
       </c>
       <c r="B40" t="s">
@@ -2110,12 +2081,12 @@
       <c r="E40" t="s">
         <v>127</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F40" s="3" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A41">
+    <row r="41" spans="1:6">
+      <c r="A41" s="1">
         <v>2019</v>
       </c>
       <c r="B41" t="s">
@@ -2130,12 +2101,12 @@
       <c r="E41" t="s">
         <v>130</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F41" s="3" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A42">
+    <row r="42" spans="1:6">
+      <c r="A42" s="1">
         <v>2018</v>
       </c>
       <c r="B42" t="s">
@@ -2150,12 +2121,12 @@
       <c r="E42" t="s">
         <v>133</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F42" s="3" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A43">
+    <row r="43" spans="1:6">
+      <c r="A43" s="1">
         <v>2018</v>
       </c>
       <c r="B43" t="s">
@@ -2170,12 +2141,12 @@
       <c r="E43" t="s">
         <v>137</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F43" s="3" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A44">
+    <row r="44" spans="1:6">
+      <c r="A44" s="1">
         <v>2018</v>
       </c>
       <c r="B44" t="s">
@@ -2190,12 +2161,12 @@
       <c r="E44" t="s">
         <v>140</v>
       </c>
-      <c r="F44" t="s">
+      <c r="F44" s="3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A45">
+    <row r="45" spans="1:6">
+      <c r="A45" s="1">
         <v>2018</v>
       </c>
       <c r="B45" t="s">
@@ -2210,12 +2181,12 @@
       <c r="E45" t="s">
         <v>143</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F45" s="3" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A46">
+    <row r="46" spans="1:6">
+      <c r="A46" s="1">
         <v>2018</v>
       </c>
       <c r="B46" t="s">
@@ -2230,12 +2201,12 @@
       <c r="E46" t="s">
         <v>146</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" s="3" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A47">
+    <row r="47" spans="1:6">
+      <c r="A47" s="1">
         <v>2017</v>
       </c>
       <c r="B47" t="s">
@@ -2250,12 +2221,12 @@
       <c r="E47" t="s">
         <v>149</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F47" s="3" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A48">
+    <row r="48" spans="1:6">
+      <c r="A48" s="1">
         <v>2017</v>
       </c>
       <c r="B48" t="s">
@@ -2270,12 +2241,12 @@
       <c r="E48" t="s">
         <v>152</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F48" s="3" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A49">
+    <row r="49" spans="1:6">
+      <c r="A49" s="1">
         <v>2017</v>
       </c>
       <c r="B49" t="s">
@@ -2290,12 +2261,12 @@
       <c r="E49" t="s">
         <v>155</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F49" s="3" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A50">
+    <row r="50" spans="1:6">
+      <c r="A50" s="1">
         <v>2017</v>
       </c>
       <c r="B50" t="s">
@@ -2310,12 +2281,12 @@
       <c r="E50" t="s">
         <v>158</v>
       </c>
-      <c r="F50" t="s">
+      <c r="F50" s="3" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A51">
+    <row r="51" spans="1:6">
+      <c r="A51" s="1">
         <v>2017</v>
       </c>
       <c r="B51" t="s">
@@ -2330,12 +2301,12 @@
       <c r="E51" t="s">
         <v>161</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F51" s="3" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A52">
+    <row r="52" spans="1:6">
+      <c r="A52" s="1">
         <v>2016</v>
       </c>
       <c r="B52" t="s">
@@ -2350,12 +2321,12 @@
       <c r="E52" t="s">
         <v>164</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F52" s="3" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A53">
+    <row r="53" spans="1:6">
+      <c r="A53" s="1">
         <v>2016</v>
       </c>
       <c r="B53" t="s">
@@ -2370,12 +2341,12 @@
       <c r="E53" t="s">
         <v>167</v>
       </c>
-      <c r="F53" t="s">
+      <c r="F53" s="3" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A54">
+    <row r="54" spans="1:6">
+      <c r="A54" s="1">
         <v>2016</v>
       </c>
       <c r="B54" t="s">
@@ -2390,12 +2361,12 @@
       <c r="E54" t="s">
         <v>170</v>
       </c>
-      <c r="F54" t="s">
+      <c r="F54" s="3" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A55">
+    <row r="55" spans="1:6">
+      <c r="A55" s="1">
         <v>2016</v>
       </c>
       <c r="B55" t="s">
@@ -2410,12 +2381,12 @@
       <c r="E55" t="s">
         <v>173</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F55" s="3" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A56">
+    <row r="56" spans="1:6">
+      <c r="A56" s="1">
         <v>2016</v>
       </c>
       <c r="B56" t="s">
@@ -2430,12 +2401,12 @@
       <c r="E56" t="s">
         <v>176</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F56" s="3" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A57">
+    <row r="57" spans="1:6">
+      <c r="A57" s="1">
         <v>2015</v>
       </c>
       <c r="B57" t="s">
@@ -2450,12 +2421,12 @@
       <c r="E57" t="s">
         <v>179</v>
       </c>
-      <c r="F57" t="s">
+      <c r="F57" s="3" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A58">
+    <row r="58" spans="1:6">
+      <c r="A58" s="1">
         <v>2015</v>
       </c>
       <c r="B58" t="s">
@@ -2470,12 +2441,12 @@
       <c r="E58" t="s">
         <v>182</v>
       </c>
-      <c r="F58" t="s">
+      <c r="F58" s="3" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A59">
+    <row r="59" spans="1:6">
+      <c r="A59" s="1">
         <v>2015</v>
       </c>
       <c r="B59" t="s">
@@ -2490,12 +2461,12 @@
       <c r="E59" t="s">
         <v>185</v>
       </c>
-      <c r="F59" t="s">
+      <c r="F59" s="3" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A60">
+    <row r="60" spans="1:6">
+      <c r="A60" s="1">
         <v>2015</v>
       </c>
       <c r="B60" t="s">
@@ -2510,12 +2481,12 @@
       <c r="E60" t="s">
         <v>188</v>
       </c>
-      <c r="F60" t="s">
+      <c r="F60" s="3" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A61">
+    <row r="61" spans="1:6">
+      <c r="A61" s="1">
         <v>2015</v>
       </c>
       <c r="B61" t="s">
@@ -2530,12 +2501,12 @@
       <c r="E61" t="s">
         <v>191</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F61" s="3" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A62">
+    <row r="62" spans="1:6">
+      <c r="A62" s="1">
         <v>2014</v>
       </c>
       <c r="B62" t="s">
@@ -2550,12 +2521,12 @@
       <c r="E62" t="s">
         <v>194</v>
       </c>
-      <c r="F62" t="s">
+      <c r="F62" s="3" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A63">
+    <row r="63" spans="1:6">
+      <c r="A63" s="1">
         <v>2014</v>
       </c>
       <c r="B63" t="s">
@@ -2570,12 +2541,12 @@
       <c r="E63" t="s">
         <v>197</v>
       </c>
-      <c r="F63" t="s">
+      <c r="F63" s="3" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A64">
+    <row r="64" spans="1:6">
+      <c r="A64" s="1">
         <v>2014</v>
       </c>
       <c r="B64" t="s">
@@ -2590,12 +2561,12 @@
       <c r="E64" t="s">
         <v>200</v>
       </c>
-      <c r="F64" t="s">
+      <c r="F64" s="3" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A65">
+    <row r="65" spans="1:6">
+      <c r="A65" s="1">
         <v>2014</v>
       </c>
       <c r="B65" t="s">
@@ -2610,12 +2581,12 @@
       <c r="E65" t="s">
         <v>203</v>
       </c>
-      <c r="F65" t="s">
+      <c r="F65" s="3" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A66">
+    <row r="66" spans="1:6">
+      <c r="A66" s="1">
         <v>2014</v>
       </c>
       <c r="B66" t="s">
@@ -2630,12 +2601,12 @@
       <c r="E66" t="s">
         <v>206</v>
       </c>
-      <c r="F66" t="s">
+      <c r="F66" s="3" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A67">
+    <row r="67" spans="1:6">
+      <c r="A67" s="1">
         <v>2013</v>
       </c>
       <c r="B67" t="s">
@@ -2650,12 +2621,12 @@
       <c r="E67" t="s">
         <v>209</v>
       </c>
-      <c r="F67" t="s">
+      <c r="F67" s="3" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A68">
+    <row r="68" spans="1:6">
+      <c r="A68" s="1">
         <v>2013</v>
       </c>
       <c r="B68" t="s">
@@ -2670,12 +2641,12 @@
       <c r="E68" t="s">
         <v>212</v>
       </c>
-      <c r="F68" t="s">
+      <c r="F68" s="3" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A69">
+    <row r="69" spans="1:6">
+      <c r="A69" s="1">
         <v>2013</v>
       </c>
       <c r="B69" t="s">
@@ -2690,12 +2661,12 @@
       <c r="E69" t="s">
         <v>215</v>
       </c>
-      <c r="F69" t="s">
+      <c r="F69" s="3" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A70">
+    <row r="70" spans="1:6">
+      <c r="A70" s="1">
         <v>2013</v>
       </c>
       <c r="B70" t="s">
@@ -2710,12 +2681,12 @@
       <c r="E70" t="s">
         <v>218</v>
       </c>
-      <c r="F70" t="s">
+      <c r="F70" s="3" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A71">
+    <row r="71" spans="1:6">
+      <c r="A71" s="1">
         <v>2013</v>
       </c>
       <c r="B71" t="s">
@@ -2730,12 +2701,12 @@
       <c r="E71" t="s">
         <v>221</v>
       </c>
-      <c r="F71" t="s">
+      <c r="F71" s="3" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A72">
+    <row r="72" spans="1:6">
+      <c r="A72" s="1">
         <v>2012</v>
       </c>
       <c r="B72" t="s">
@@ -2750,12 +2721,12 @@
       <c r="E72" t="s">
         <v>224</v>
       </c>
-      <c r="F72" t="s">
+      <c r="F72" s="3" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A73">
+    <row r="73" spans="1:6">
+      <c r="A73" s="1">
         <v>2012</v>
       </c>
       <c r="B73" t="s">
@@ -2770,12 +2741,12 @@
       <c r="E73" t="s">
         <v>227</v>
       </c>
-      <c r="F73" t="s">
+      <c r="F73" s="3" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A74">
+    <row r="74" spans="1:6">
+      <c r="A74" s="1">
         <v>2012</v>
       </c>
       <c r="B74" t="s">
@@ -2790,12 +2761,12 @@
       <c r="E74" t="s">
         <v>230</v>
       </c>
-      <c r="F74" t="s">
+      <c r="F74" s="3" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A75">
+    <row r="75" spans="1:6">
+      <c r="A75" s="1">
         <v>2012</v>
       </c>
       <c r="B75" t="s">
@@ -2810,12 +2781,12 @@
       <c r="E75" t="s">
         <v>233</v>
       </c>
-      <c r="F75" t="s">
+      <c r="F75" s="3" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A76">
+    <row r="76" spans="1:6">
+      <c r="A76" s="1">
         <v>2012</v>
       </c>
       <c r="B76" t="s">
@@ -2830,12 +2801,12 @@
       <c r="E76" t="s">
         <v>236</v>
       </c>
-      <c r="F76" t="s">
+      <c r="F76" s="3" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A77">
+    <row r="77" spans="1:6">
+      <c r="A77" s="1">
         <v>2011</v>
       </c>
       <c r="B77" t="s">
@@ -2850,12 +2821,12 @@
       <c r="E77" t="s">
         <v>239</v>
       </c>
-      <c r="F77" t="s">
+      <c r="F77" s="3" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A78">
+    <row r="78" spans="1:6">
+      <c r="A78" s="1">
         <v>2011</v>
       </c>
       <c r="B78" t="s">
@@ -2870,12 +2841,12 @@
       <c r="E78" t="s">
         <v>242</v>
       </c>
-      <c r="F78" t="s">
+      <c r="F78" s="3" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A79">
+    <row r="79" spans="1:6">
+      <c r="A79" s="1">
         <v>2011</v>
       </c>
       <c r="B79" t="s">
@@ -2890,12 +2861,12 @@
       <c r="E79" t="s">
         <v>245</v>
       </c>
-      <c r="F79" t="s">
+      <c r="F79" s="3" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A80">
+    <row r="80" spans="1:6">
+      <c r="A80" s="1">
         <v>2011</v>
       </c>
       <c r="B80" t="s">
@@ -2910,12 +2881,12 @@
       <c r="E80" t="s">
         <v>248</v>
       </c>
-      <c r="F80" t="s">
+      <c r="F80" s="3" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A81">
+    <row r="81" spans="1:6">
+      <c r="A81" s="1">
         <v>2011</v>
       </c>
       <c r="B81" t="s">
@@ -2930,12 +2901,12 @@
       <c r="E81" t="s">
         <v>251</v>
       </c>
-      <c r="F81" t="s">
+      <c r="F81" s="3" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A82">
+    <row r="82" spans="1:6">
+      <c r="A82" s="1">
         <v>2010</v>
       </c>
       <c r="B82" t="s">
@@ -2950,12 +2921,12 @@
       <c r="E82" t="s">
         <v>254</v>
       </c>
-      <c r="F82" t="s">
+      <c r="F82" s="3" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A83">
+    <row r="83" spans="1:6">
+      <c r="A83" s="1">
         <v>2010</v>
       </c>
       <c r="B83" t="s">
@@ -2970,12 +2941,12 @@
       <c r="E83" t="s">
         <v>257</v>
       </c>
-      <c r="F83" t="s">
+      <c r="F83" s="3" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A84">
+    <row r="84" spans="1:6">
+      <c r="A84" s="1">
         <v>2010</v>
       </c>
       <c r="B84" t="s">
@@ -2990,12 +2961,12 @@
       <c r="E84" t="s">
         <v>260</v>
       </c>
-      <c r="F84" t="s">
+      <c r="F84" s="3" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A85">
+    <row r="85" spans="1:6">
+      <c r="A85" s="1">
         <v>2010</v>
       </c>
       <c r="B85" t="s">
@@ -3010,12 +2981,12 @@
       <c r="E85" t="s">
         <v>263</v>
       </c>
-      <c r="F85" t="s">
+      <c r="F85" s="3" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A86">
+    <row r="86" spans="1:6">
+      <c r="A86" s="1">
         <v>2010</v>
       </c>
       <c r="B86" t="s">
@@ -3030,12 +3001,12 @@
       <c r="E86" t="s">
         <v>266</v>
       </c>
-      <c r="F86" t="s">
+      <c r="F86" s="3" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A87">
+    <row r="87" spans="1:6">
+      <c r="A87" s="1">
         <v>2009</v>
       </c>
       <c r="B87" t="s">
@@ -3050,12 +3021,12 @@
       <c r="E87" t="s">
         <v>269</v>
       </c>
-      <c r="F87" t="s">
+      <c r="F87" s="3" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A88">
+    <row r="88" spans="1:6">
+      <c r="A88" s="1">
         <v>2009</v>
       </c>
       <c r="B88" t="s">
@@ -3070,12 +3041,12 @@
       <c r="E88" t="s">
         <v>272</v>
       </c>
-      <c r="F88" t="s">
+      <c r="F88" s="3" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A89">
+    <row r="89" spans="1:6">
+      <c r="A89" s="1">
         <v>2009</v>
       </c>
       <c r="B89" t="s">
@@ -3090,12 +3061,12 @@
       <c r="E89" t="s">
         <v>275</v>
       </c>
-      <c r="F89" t="s">
+      <c r="F89" s="3" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A90">
+    <row r="90" spans="1:6">
+      <c r="A90" s="1">
         <v>2009</v>
       </c>
       <c r="B90" t="s">
@@ -3110,12 +3081,12 @@
       <c r="E90" t="s">
         <v>278</v>
       </c>
-      <c r="F90" t="s">
+      <c r="F90" s="3" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A91">
+    <row r="91" spans="1:6">
+      <c r="A91" s="1">
         <v>2009</v>
       </c>
       <c r="B91" t="s">
@@ -3130,12 +3101,12 @@
       <c r="E91" t="s">
         <v>281</v>
       </c>
-      <c r="F91" t="s">
+      <c r="F91" s="3" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A92">
+    <row r="92" spans="1:6">
+      <c r="A92" s="1">
         <v>2008</v>
       </c>
       <c r="B92" t="s">
@@ -3150,12 +3121,12 @@
       <c r="E92" t="s">
         <v>284</v>
       </c>
-      <c r="F92" t="s">
+      <c r="F92" s="3" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A93">
+    <row r="93" spans="1:6">
+      <c r="A93" s="1">
         <v>2008</v>
       </c>
       <c r="B93" t="s">
@@ -3170,12 +3141,12 @@
       <c r="E93" t="s">
         <v>287</v>
       </c>
-      <c r="F93" t="s">
+      <c r="F93" s="3" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A94">
+    <row r="94" spans="1:6">
+      <c r="A94" s="1">
         <v>2008</v>
       </c>
       <c r="B94" t="s">
@@ -3190,12 +3161,12 @@
       <c r="E94" t="s">
         <v>290</v>
       </c>
-      <c r="F94" t="s">
+      <c r="F94" s="3" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A95">
+    <row r="95" spans="1:6">
+      <c r="A95" s="1">
         <v>2008</v>
       </c>
       <c r="B95" t="s">
@@ -3210,12 +3181,12 @@
       <c r="E95" t="s">
         <v>293</v>
       </c>
-      <c r="F95" t="s">
+      <c r="F95" s="3" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A96">
+    <row r="96" spans="1:6">
+      <c r="A96" s="1">
         <v>2008</v>
       </c>
       <c r="B96" t="s">
@@ -3230,12 +3201,111 @@
       <c r="E96" t="s">
         <v>296</v>
       </c>
-      <c r="F96" t="s">
+      <c r="F96" s="3" t="s">
         <v>297</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F96" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1"/>
+    <hyperlink ref="F3" r:id="rId2"/>
+    <hyperlink ref="F4" r:id="rId3"/>
+    <hyperlink ref="F5" r:id="rId4"/>
+    <hyperlink ref="F6" r:id="rId5"/>
+    <hyperlink ref="F7" r:id="rId6"/>
+    <hyperlink ref="F8" r:id="rId7"/>
+    <hyperlink ref="F9" r:id="rId8"/>
+    <hyperlink ref="F10" r:id="rId9"/>
+    <hyperlink ref="F11" r:id="rId10"/>
+    <hyperlink ref="F12" r:id="rId11"/>
+    <hyperlink ref="F13" r:id="rId12"/>
+    <hyperlink ref="F14" r:id="rId13"/>
+    <hyperlink ref="F15" r:id="rId14"/>
+    <hyperlink ref="F16" r:id="rId15"/>
+    <hyperlink ref="F17" r:id="rId16"/>
+    <hyperlink ref="F18" r:id="rId17"/>
+    <hyperlink ref="F19" r:id="rId18"/>
+    <hyperlink ref="F20" r:id="rId19"/>
+    <hyperlink ref="F21" r:id="rId20"/>
+    <hyperlink ref="F22" r:id="rId21"/>
+    <hyperlink ref="F23" r:id="rId22"/>
+    <hyperlink ref="F24" r:id="rId23"/>
+    <hyperlink ref="F25" r:id="rId24"/>
+    <hyperlink ref="F26" r:id="rId25"/>
+    <hyperlink ref="F27" r:id="rId26"/>
+    <hyperlink ref="F28" r:id="rId27"/>
+    <hyperlink ref="F29" r:id="rId28"/>
+    <hyperlink ref="F30" r:id="rId29"/>
+    <hyperlink ref="F31" r:id="rId30"/>
+    <hyperlink ref="F32" r:id="rId31"/>
+    <hyperlink ref="F33" r:id="rId32"/>
+    <hyperlink ref="F34" r:id="rId33"/>
+    <hyperlink ref="F35" r:id="rId34"/>
+    <hyperlink ref="F36" r:id="rId35"/>
+    <hyperlink ref="F37" r:id="rId36"/>
+    <hyperlink ref="F38" r:id="rId37"/>
+    <hyperlink ref="F39" r:id="rId38"/>
+    <hyperlink ref="F40" r:id="rId39"/>
+    <hyperlink ref="F41" r:id="rId40"/>
+    <hyperlink ref="F42" r:id="rId41"/>
+    <hyperlink ref="F43" r:id="rId42"/>
+    <hyperlink ref="F44" r:id="rId43"/>
+    <hyperlink ref="F45" r:id="rId44"/>
+    <hyperlink ref="F46" r:id="rId45"/>
+    <hyperlink ref="F47" r:id="rId46"/>
+    <hyperlink ref="F48" r:id="rId47"/>
+    <hyperlink ref="F49" r:id="rId48"/>
+    <hyperlink ref="F50" r:id="rId49"/>
+    <hyperlink ref="F51" r:id="rId50"/>
+    <hyperlink ref="F52" r:id="rId51"/>
+    <hyperlink ref="F53" r:id="rId52"/>
+    <hyperlink ref="F54" r:id="rId53"/>
+    <hyperlink ref="F55" r:id="rId54"/>
+    <hyperlink ref="F56" r:id="rId55"/>
+    <hyperlink ref="F57" r:id="rId56"/>
+    <hyperlink ref="F58" r:id="rId57"/>
+    <hyperlink ref="F59" r:id="rId58"/>
+    <hyperlink ref="F60" r:id="rId59"/>
+    <hyperlink ref="F61" r:id="rId60"/>
+    <hyperlink ref="F62" r:id="rId61"/>
+    <hyperlink ref="F63" r:id="rId62"/>
+    <hyperlink ref="F64" r:id="rId63"/>
+    <hyperlink ref="F65" r:id="rId64"/>
+    <hyperlink ref="F66" r:id="rId65"/>
+    <hyperlink ref="F67" r:id="rId66"/>
+    <hyperlink ref="F68" r:id="rId67"/>
+    <hyperlink ref="F69" r:id="rId68"/>
+    <hyperlink ref="F70" r:id="rId69"/>
+    <hyperlink ref="F71" r:id="rId70"/>
+    <hyperlink ref="F72" r:id="rId71"/>
+    <hyperlink ref="F73" r:id="rId72"/>
+    <hyperlink ref="F74" r:id="rId73"/>
+    <hyperlink ref="F75" r:id="rId74"/>
+    <hyperlink ref="F76" r:id="rId75"/>
+    <hyperlink ref="F77" r:id="rId76"/>
+    <hyperlink ref="F78" r:id="rId77"/>
+    <hyperlink ref="F79" r:id="rId78"/>
+    <hyperlink ref="F80" r:id="rId79"/>
+    <hyperlink ref="F81" r:id="rId80"/>
+    <hyperlink ref="F82" r:id="rId81"/>
+    <hyperlink ref="F83" r:id="rId82"/>
+    <hyperlink ref="F84" r:id="rId83"/>
+    <hyperlink ref="F85" r:id="rId84"/>
+    <hyperlink ref="F86" r:id="rId85"/>
+    <hyperlink ref="F87" r:id="rId86"/>
+    <hyperlink ref="F88" r:id="rId87"/>
+    <hyperlink ref="F89" r:id="rId88"/>
+    <hyperlink ref="F90" r:id="rId89"/>
+    <hyperlink ref="F91" r:id="rId90"/>
+    <hyperlink ref="F92" r:id="rId91"/>
+    <hyperlink ref="F93" r:id="rId92"/>
+    <hyperlink ref="F94" r:id="rId93"/>
+    <hyperlink ref="F95" r:id="rId94"/>
+    <hyperlink ref="F96" r:id="rId95"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId96"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>